<commit_message>
Down-sampling to 200 Hz
</commit_message>
<xml_diff>
--- a/arousal_annotations.xlsx
+++ b/arousal_annotations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/barbora/Projekty/arousal/Sana/nature_submission_code/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\ANPHY2\Workspace\Barbora\Hannan_code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E6A3C27-F55B-D14C-919E-33CCDE3878A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F4AD131-D84F-4353-B2F5-1348239E9907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16280" xr2:uid="{EAE4818D-61D2-3F41-9500-CBA7F81496B9}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="12645" xr2:uid="{EAE4818D-61D2-3F41-9500-CBA7F81496B9}"/>
   </bookViews>
   <sheets>
     <sheet name="stimulations" sheetId="1" r:id="rId1"/>
@@ -99,7 +99,7 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normální" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -115,7 +115,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Motiv Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -431,16 +431,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2CFEF45-38D6-CE45-9060-676BDADC16CC}">
-  <dimension ref="A1:H21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="12.6640625" customWidth="1"/>
-    <col min="6" max="6" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.625" customWidth="1"/>
+    <col min="6" max="6" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -451,255 +451,255 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>125100</v>
+        <v>12217</v>
       </c>
       <c r="C2">
-        <v>125677</v>
-      </c>
+        <v>12273</v>
+      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3">
-        <v>644171</v>
+        <v>62907</v>
       </c>
       <c r="C3">
-        <v>644514</v>
-      </c>
+        <v>62941</v>
+      </c>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
       <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4">
-        <v>903645</v>
+        <v>88247</v>
       </c>
       <c r="C4">
-        <v>903887</v>
-      </c>
+        <v>88270</v>
+      </c>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>0</v>
       </c>
       <c r="B5">
-        <v>1163161</v>
+        <v>113590</v>
       </c>
       <c r="C5">
-        <v>1171830</v>
-      </c>
+        <v>114437</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
       <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>0</v>
       </c>
       <c r="B6">
-        <v>1422505</v>
+        <v>138917</v>
       </c>
       <c r="C6">
-        <v>1422859</v>
-      </c>
+        <v>138951</v>
+      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>0</v>
       </c>
       <c r="B7">
-        <v>2534397</v>
-      </c>
+        <v>247500</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>0</v>
       </c>
       <c r="B8">
-        <v>2793971</v>
-      </c>
+        <v>272849</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>0</v>
       </c>
       <c r="B9">
-        <v>2836103</v>
-      </c>
+        <v>276963</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
       <c r="B10">
-        <v>2848421</v>
-      </c>
+        <v>278166</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>0</v>
       </c>
       <c r="B11">
-        <v>2869721</v>
-      </c>
+        <v>280246</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>1</v>
       </c>
       <c r="B12">
-        <v>63401</v>
-      </c>
+        <v>6192</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>1</v>
       </c>
       <c r="B13">
-        <v>217806</v>
-      </c>
+        <v>21270</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>1</v>
       </c>
       <c r="B14">
-        <v>477276</v>
-      </c>
+        <v>46609</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>1</v>
       </c>
       <c r="B15">
-        <v>736571</v>
+        <v>71931</v>
       </c>
       <c r="C15">
-        <v>738129</v>
-      </c>
+        <v>72083</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>1</v>
       </c>
       <c r="B16">
-        <v>995854</v>
+        <v>97251</v>
       </c>
       <c r="C16">
-        <v>997329</v>
-      </c>
+        <v>97395</v>
+      </c>
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>1</v>
       </c>
       <c r="B17">
-        <v>1255313</v>
-      </c>
+        <v>122589</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
       <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>1</v>
       </c>
       <c r="B18">
-        <v>1514635</v>
+        <v>147914</v>
       </c>
       <c r="C18">
-        <v>1515766</v>
-      </c>
+        <v>148024</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
       <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>1</v>
       </c>
       <c r="B19">
-        <v>1774120</v>
-      </c>
+        <v>173254</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
       <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>1</v>
       </c>
       <c r="B20">
-        <v>2033338</v>
+        <v>198568</v>
       </c>
       <c r="C20">
-        <v>2035218</v>
-      </c>
+        <v>198752</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
       <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>1</v>
       </c>
       <c r="B21">
-        <v>2676023</v>
+        <v>261330</v>
       </c>
       <c r="C21">
-        <v>2677365</v>
-      </c>
+        <v>261461</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
       <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
New version after reviews
Updated code according to Nature Communications review comments
</commit_message>
<xml_diff>
--- a/arousal_annotations.xlsx
+++ b/arousal_annotations.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\ANPHY2\Workspace\Barbora\Hannan_code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/barbora/Projekty/arousal/Sana/nature_submission_code/Hannan_code_v2/Hannan_code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F4AD131-D84F-4353-B2F5-1348239E9907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3B54EC84-E82F-0749-95B1-DE1927D2F575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="1125" windowWidth="21600" windowHeight="12645" xr2:uid="{EAE4818D-61D2-3F41-9500-CBA7F81496B9}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16340" xr2:uid="{1C57E1CA-41C2-784E-BEB0-66F8B443A3A3}"/>
   </bookViews>
   <sheets>
-    <sheet name="stimulations" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -31,44 +31,90 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="22">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>stim_intensity</t>
+  </si>
+  <si>
+    <t>utc_stim_start</t>
+  </si>
+  <si>
+    <t>utc_arousal_start</t>
+  </si>
+  <si>
+    <t>arousal_duration</t>
+  </si>
+  <si>
+    <t>stage</t>
+  </si>
+  <si>
+    <t>stage_post</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
   <si>
     <t>P11</t>
   </si>
   <si>
+    <t>AudioStim 90</t>
+  </si>
+  <si>
+    <t>N2</t>
+  </si>
+  <si>
+    <t>control</t>
+  </si>
+  <si>
+    <t>N3</t>
+  </si>
+  <si>
+    <t>spontaneous</t>
+  </si>
+  <si>
+    <t>evoked</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
     <t>P14</t>
   </si>
   <si>
-    <t>stim_start</t>
-  </si>
-  <si>
-    <t>arousal_start</t>
-  </si>
-  <si>
-    <t>patient</t>
+    <t>AudioStim 80</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>N1</t>
+  </si>
+  <si>
+    <t>AudioStim 70</t>
+  </si>
+  <si>
+    <t>AudioStim 40</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <charset val="238"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -94,9 +140,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -430,279 +475,401 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2CFEF45-38D6-CE45-9060-676BDADC16CC}">
-  <dimension ref="A1:F21"/>
-  <sheetFormatPr defaultColWidth="11.5" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C41FE555-FEDA-DB47-B222-B99529093C07}">
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="12.625" customWidth="1"/>
-    <col min="6" max="6" width="11.125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.625" customWidth="1"/>
+    <col min="2" max="2" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2">
-        <v>12217</v>
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
       </c>
       <c r="C2">
-        <v>12273</v>
-      </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1704770210.36572</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3">
-        <v>62907</v>
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
       </c>
       <c r="C3">
-        <v>62941</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1704770336.97753</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4">
-        <v>88247</v>
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
       </c>
       <c r="C4">
-        <v>88270</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1704770463.5527301</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5">
-        <v>113590</v>
-      </c>
-      <c r="C5">
-        <v>114437</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>1704770557.6166899</v>
+      </c>
+      <c r="E5">
+        <v>4.88671875</v>
+      </c>
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6">
-        <v>138917</v>
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
       </c>
       <c r="C6">
-        <v>138951</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1704770590.2509699</v>
+      </c>
+      <c r="D6">
+        <v>1704770591.3808501</v>
+      </c>
+      <c r="E6">
+        <v>9.70703125</v>
+      </c>
+      <c r="F6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7">
-        <v>247500</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7">
+        <v>1704770716.9589801</v>
+      </c>
+      <c r="D7">
+        <v>1704770721.06494</v>
+      </c>
+      <c r="E7">
+        <v>3.7421875</v>
+      </c>
+      <c r="F7" t="s">
+        <v>10</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8">
-        <v>272849</v>
-      </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8">
+        <v>1704770843.6396401</v>
+      </c>
+      <c r="D8">
+        <v>1704770844.23437</v>
+      </c>
+      <c r="E8">
+        <v>12.98681640625</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B9">
-        <v>276963</v>
-      </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>1704770905.1591699</v>
+      </c>
+      <c r="E9">
+        <v>13.646484375</v>
+      </c>
+      <c r="F9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10">
-        <v>278166</v>
-      </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>1719360902.3496001</v>
+      </c>
+      <c r="D10">
+        <v>1719360903.4208901</v>
+      </c>
+      <c r="E10">
+        <v>14.494140625</v>
+      </c>
+      <c r="F10" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11">
-        <v>280246</v>
-      </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11">
+        <v>1719360990.3867099</v>
+      </c>
+      <c r="F11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>1</v>
-      </c>
-      <c r="B12">
-        <v>6192</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="D12">
+        <v>1719361088.4624</v>
+      </c>
+      <c r="E12">
+        <v>4.6591796875</v>
+      </c>
+      <c r="F12" t="s">
+        <v>10</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13">
-        <v>21270</v>
-      </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13">
+        <v>1719361117.04882</v>
+      </c>
+      <c r="D13">
+        <v>1719361117.9448199</v>
+      </c>
+      <c r="E13">
+        <v>5.1318359375</v>
+      </c>
+      <c r="F13" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" t="s">
+        <v>10</v>
+      </c>
+      <c r="H13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14">
-        <v>46609</v>
-      </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="B14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14">
+        <v>1719361243.7465799</v>
+      </c>
+      <c r="F14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+      <c r="H14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B15">
-        <v>71931</v>
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>9</v>
       </c>
       <c r="C15">
-        <v>72083</v>
-      </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+        <v>1719361370.4716699</v>
+      </c>
+      <c r="D15">
+        <v>1719361371.22314</v>
+      </c>
+      <c r="E15">
+        <v>7.98974609375</v>
+      </c>
+      <c r="F15" t="s">
+        <v>10</v>
+      </c>
+      <c r="G15" t="s">
+        <v>18</v>
+      </c>
+      <c r="H15" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>1</v>
-      </c>
-      <c r="B16">
-        <v>97251</v>
-      </c>
-      <c r="C16">
-        <v>97395</v>
-      </c>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="D16">
+        <v>1719361638.4545801</v>
+      </c>
+      <c r="E16">
+        <v>10.9833984375</v>
+      </c>
+      <c r="F16" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" t="s">
+        <v>18</v>
+      </c>
+      <c r="H16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>1</v>
-      </c>
-      <c r="B17">
-        <v>122589</v>
-      </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18">
-        <v>147914</v>
-      </c>
-      <c r="C18">
-        <v>148024</v>
-      </c>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19">
-        <v>173254</v>
-      </c>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>1</v>
-      </c>
-      <c r="B20">
-        <v>198568</v>
-      </c>
-      <c r="C20">
-        <v>198752</v>
-      </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21">
-        <v>261330</v>
-      </c>
-      <c r="C21">
-        <v>261461</v>
-      </c>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17">
+        <v>1719361948.1166899</v>
+      </c>
+      <c r="F17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" t="s">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>